<commit_message>
20 05 26 17 14й
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967F8C72-7C2B-4192-9451-56C16D874BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9017C36F-765D-41D8-A342-187728F7FDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_helper" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2752" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2597" uniqueCount="134">
   <si>
     <t>id</t>
   </si>
@@ -425,6 +425,45 @@
   </si>
   <si>
     <t>card1</t>
+  </si>
+  <si>
+    <r>
+      <t>Заживление пигмента в коже</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Во время процедуры игла вводит пигмент в верхние слои дермы — не слишком глубоко, но и не в эпидермис, иначе пигмент уйдёт вместе с шелушением кожи за 3–4 недели; во время проколов кожа воспринимает процедуру как микротравму.</t>
+  </si>
+  <si>
+    <t>повреждаются мелкие сосуды,</t>
+  </si>
+  <si>
+    <t>выделяется лимфа,</t>
+  </si>
+  <si>
+    <t>запускается воспалительная реакция и заживление.</t>
+  </si>
+  <si>
+    <t>ярче,</t>
+  </si>
+  <si>
+    <t>плотнее,</t>
+  </si>
+  <si>
+    <t>темнее.</t>
+  </si>
+  <si>
+    <t>Сразу после процедуры цвет выглядит</t>
   </si>
 </sst>
 </file>
@@ -23258,7 +23297,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90F4ED04-88E6-4270-B7F6-4E9A515B69D3}">
-  <dimension ref="A1:P165"/>
+  <dimension ref="A1:P126"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.875" bestFit="1" customWidth="1"/>
@@ -23354,39 +23393,39 @@
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" ht="15">
       <c r="A3" s="6">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="6">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0</v>
+        <v>125</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
@@ -23395,37 +23434,37 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="6">
-        <v>3</v>
+        <v>43</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
@@ -23434,20 +23473,38 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="6">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
+        <v>68</v>
+      </c>
+      <c r="C5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>123</v>
+      </c>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -23455,74 +23512,76 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="6">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>123</v>
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" t="s">
+        <v>128</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>88</v>
+        <v>123</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>123</v>
+      </c>
       <c r="K6" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="L6" s="6">
-        <v>600</v>
-      </c>
-      <c r="M6" s="6">
-        <v>600</v>
-      </c>
-      <c r="N6" s="6">
-        <v>1</v>
-      </c>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="6">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="C7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -23531,37 +23590,37 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="6">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E8" s="6">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0</v>
-      </c>
-      <c r="K8" s="6">
-        <v>0</v>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
@@ -23570,37 +23629,37 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="6">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0</v>
-      </c>
-      <c r="H9" s="6">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>0</v>
+      <c r="C9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
@@ -23609,37 +23668,37 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" s="6">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6">
-        <v>0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>0</v>
+      <c r="C10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K10" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
@@ -23648,37 +23707,37 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="6">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6">
-        <v>0</v>
+      <c r="C11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K11" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
@@ -23687,37 +23746,35 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="6">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0</v>
-      </c>
-      <c r="H12" s="6">
-        <v>0</v>
+        <v>51</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K12" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
@@ -23726,37 +23783,35 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="6">
-        <v>12</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>0</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K13" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
@@ -23765,37 +23820,35 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="6">
-        <v>13</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6">
-        <v>0</v>
-      </c>
-      <c r="K14" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L14" s="6"/>
       <c r="M14" s="6"/>
@@ -23804,37 +23857,35 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="6">
-        <v>14</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>24</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B15" s="6"/>
       <c r="C15" s="6" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E15" s="6">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0</v>
-      </c>
-      <c r="H15" s="6">
-        <v>0</v>
-      </c>
-      <c r="I15" s="6">
-        <v>0</v>
-      </c>
-      <c r="J15" s="6">
-        <v>0</v>
-      </c>
-      <c r="K15" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L15" s="6"/>
       <c r="M15" s="6"/>
@@ -23843,37 +23894,35 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="6">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B16" s="6"/>
       <c r="C16" s="6" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0</v>
-      </c>
-      <c r="F16" s="6">
-        <v>0</v>
-      </c>
-      <c r="G16" s="6">
-        <v>0</v>
-      </c>
-      <c r="H16" s="6">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6">
-        <v>0</v>
-      </c>
-      <c r="J16" s="6">
-        <v>0</v>
-      </c>
-      <c r="K16" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L16" s="6"/>
       <c r="M16" s="6"/>
@@ -23882,37 +23931,35 @@
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="6">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B17" s="6"/>
       <c r="C17" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E17" s="6">
-        <v>0</v>
-      </c>
-      <c r="F17" s="6">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K17" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
@@ -23921,37 +23968,35 @@
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="6">
-        <v>17</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="B18" s="6"/>
       <c r="C18" s="6" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E18" s="6">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>0</v>
-      </c>
-      <c r="H18" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K18" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L18" s="6"/>
       <c r="M18" s="6"/>
@@ -23960,37 +24005,35 @@
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="6">
-        <v>18</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B19" s="6"/>
       <c r="C19" s="6" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E19" s="6">
-        <v>0</v>
-      </c>
-      <c r="F19" s="6">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6">
-        <v>0</v>
-      </c>
-      <c r="H19" s="6">
-        <v>0</v>
-      </c>
-      <c r="I19" s="6">
-        <v>0</v>
-      </c>
-      <c r="J19" s="6">
-        <v>0</v>
-      </c>
-      <c r="K19" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
@@ -23999,37 +24042,35 @@
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="6">
-        <v>19</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B20" s="6"/>
       <c r="C20" s="6" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E20" s="6">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6">
-        <v>0</v>
-      </c>
-      <c r="H20" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K20" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L20" s="6"/>
       <c r="M20" s="6"/>
@@ -24038,37 +24079,35 @@
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="6">
-        <v>20</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="B21" s="6"/>
       <c r="C21" s="6" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E21" s="6">
-        <v>0</v>
-      </c>
-      <c r="F21" s="6">
-        <v>0</v>
-      </c>
-      <c r="G21" s="6">
-        <v>0</v>
-      </c>
-      <c r="H21" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K21" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
@@ -24077,37 +24116,35 @@
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="6">
-        <v>21</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="B22" s="6"/>
       <c r="C22" s="6" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="E22" s="6">
-        <v>0</v>
-      </c>
-      <c r="F22" s="6">
-        <v>0</v>
-      </c>
-      <c r="G22" s="6">
-        <v>0</v>
-      </c>
-      <c r="H22" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K22" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
@@ -24116,37 +24153,35 @@
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="6">
-        <v>22</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="B23" s="6"/>
       <c r="C23" s="6" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E23" s="6">
-        <v>0</v>
-      </c>
-      <c r="F23" s="6">
-        <v>0</v>
-      </c>
-      <c r="G23" s="6">
-        <v>0</v>
-      </c>
-      <c r="H23" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K23" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
@@ -24155,37 +24190,35 @@
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="6">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="B24" s="6"/>
       <c r="C24" s="6" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E24" s="6">
-        <v>0</v>
-      </c>
-      <c r="F24" s="6">
-        <v>0</v>
-      </c>
-      <c r="G24" s="6">
-        <v>0</v>
-      </c>
-      <c r="H24" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K24" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
@@ -24194,37 +24227,35 @@
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="6">
-        <v>24</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="B25" s="6"/>
       <c r="C25" s="6" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="E25" s="6">
-        <v>0</v>
-      </c>
-      <c r="F25" s="6">
-        <v>0</v>
-      </c>
-      <c r="G25" s="6">
-        <v>0</v>
-      </c>
-      <c r="H25" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K25" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
@@ -24233,37 +24264,35 @@
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="6">
-        <v>25</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E26" s="6">
-        <v>0</v>
-      </c>
-      <c r="F26" s="6">
-        <v>0</v>
-      </c>
-      <c r="G26" s="6">
-        <v>0</v>
-      </c>
-      <c r="H26" s="6">
-        <v>0</v>
-      </c>
-      <c r="I26" s="6">
-        <v>0</v>
-      </c>
-      <c r="J26" s="6">
-        <v>0</v>
-      </c>
-      <c r="K26" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L26" s="6"/>
       <c r="M26" s="6"/>
@@ -24272,37 +24301,35 @@
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="6">
-        <v>26</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="6">
-        <v>0</v>
-      </c>
-      <c r="F27" s="6">
-        <v>0</v>
-      </c>
-      <c r="G27" s="6">
-        <v>0</v>
-      </c>
-      <c r="H27" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K27" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
@@ -24311,37 +24338,35 @@
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="6">
-        <v>27</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" s="6">
-        <v>0</v>
-      </c>
-      <c r="F28" s="6">
-        <v>0</v>
-      </c>
-      <c r="G28" s="6">
-        <v>0</v>
-      </c>
-      <c r="H28" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K28" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
@@ -24350,37 +24375,35 @@
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="6">
-        <v>28</v>
-      </c>
-      <c r="B29" s="6" t="s">
         <v>68</v>
       </c>
+      <c r="B29" s="6"/>
       <c r="C29" s="6" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="E29" s="6">
-        <v>0</v>
-      </c>
-      <c r="F29" s="6">
-        <v>0</v>
-      </c>
-      <c r="G29" s="6">
-        <v>0</v>
-      </c>
-      <c r="H29" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K29" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
@@ -24389,37 +24412,35 @@
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="6">
-        <v>29</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>24</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="B30" s="6"/>
       <c r="C30" s="6" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E30" s="6">
-        <v>0</v>
-      </c>
-      <c r="F30" s="6">
-        <v>0</v>
-      </c>
-      <c r="G30" s="6">
-        <v>0</v>
-      </c>
-      <c r="H30" s="6">
-        <v>0</v>
-      </c>
-      <c r="I30" s="6">
-        <v>0</v>
-      </c>
-      <c r="J30" s="6">
-        <v>0</v>
-      </c>
-      <c r="K30" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L30" s="6"/>
       <c r="M30" s="6"/>
@@ -24428,37 +24449,35 @@
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="6">
-        <v>30</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="B31" s="6"/>
       <c r="C31" s="6" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="E31" s="6">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6">
-        <v>0</v>
-      </c>
-      <c r="G31" s="6">
-        <v>0</v>
-      </c>
-      <c r="H31" s="6">
-        <v>0</v>
-      </c>
-      <c r="I31" s="6">
-        <v>0</v>
-      </c>
-      <c r="J31" s="6">
-        <v>0</v>
-      </c>
-      <c r="K31" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
@@ -24467,37 +24486,35 @@
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="6">
-        <v>31</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="B32" s="6"/>
       <c r="C32" s="6" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="E32" s="6">
-        <v>0</v>
-      </c>
-      <c r="F32" s="6">
-        <v>0</v>
-      </c>
-      <c r="G32" s="6">
-        <v>0</v>
-      </c>
-      <c r="H32" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K32" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L32" s="6"/>
       <c r="M32" s="6"/>
@@ -24506,37 +24523,35 @@
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="6">
-        <v>32</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="B33" s="6"/>
       <c r="C33" s="6" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="E33" s="6">
-        <v>0</v>
-      </c>
-      <c r="F33" s="6">
-        <v>0</v>
-      </c>
-      <c r="G33" s="6">
-        <v>0</v>
-      </c>
-      <c r="H33" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K33" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
@@ -24545,37 +24560,35 @@
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="6">
-        <v>33</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="B34" s="6"/>
       <c r="C34" s="6" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="E34" s="6">
-        <v>0</v>
-      </c>
-      <c r="F34" s="6">
-        <v>0</v>
-      </c>
-      <c r="G34" s="6">
-        <v>0</v>
-      </c>
-      <c r="H34" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K34" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L34" s="6"/>
       <c r="M34" s="6"/>
@@ -24584,37 +24597,35 @@
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="6">
-        <v>34</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="B35" s="6"/>
       <c r="C35" s="6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E35" s="6">
-        <v>0</v>
-      </c>
-      <c r="F35" s="6">
-        <v>0</v>
-      </c>
-      <c r="G35" s="6">
-        <v>0</v>
-      </c>
-      <c r="H35" s="6">
-        <v>0</v>
-      </c>
-      <c r="I35" s="6">
-        <v>0</v>
-      </c>
-      <c r="J35" s="6">
-        <v>0</v>
-      </c>
-      <c r="K35" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
@@ -24623,37 +24634,35 @@
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="6">
-        <v>35</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="B36" s="6"/>
       <c r="C36" s="6" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="E36" s="6">
-        <v>0</v>
-      </c>
-      <c r="F36" s="6">
-        <v>0</v>
-      </c>
-      <c r="G36" s="6">
-        <v>0</v>
-      </c>
-      <c r="H36" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K36" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L36" s="6"/>
       <c r="M36" s="6"/>
@@ -24662,37 +24671,35 @@
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="6">
-        <v>36</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="B37" s="6"/>
       <c r="C37" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E37" s="6">
-        <v>0</v>
-      </c>
-      <c r="F37" s="6">
-        <v>0</v>
-      </c>
-      <c r="G37" s="6">
-        <v>0</v>
-      </c>
-      <c r="H37" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K37" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
@@ -24701,37 +24708,35 @@
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="6">
-        <v>37</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="B38" s="6"/>
       <c r="C38" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="E38" s="6">
-        <v>0</v>
-      </c>
-      <c r="F38" s="6">
-        <v>0</v>
-      </c>
-      <c r="G38" s="6">
-        <v>0</v>
-      </c>
-      <c r="H38" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K38" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L38" s="6"/>
       <c r="M38" s="6"/>
@@ -24740,37 +24745,35 @@
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="6">
-        <v>38</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="B39" s="6"/>
       <c r="C39" s="6" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E39" s="6">
-        <v>0</v>
-      </c>
-      <c r="F39" s="6">
-        <v>0</v>
-      </c>
-      <c r="G39" s="6">
-        <v>0</v>
-      </c>
-      <c r="H39" s="6">
-        <v>0</v>
-      </c>
-      <c r="I39" s="6">
-        <v>0</v>
-      </c>
-      <c r="J39" s="6">
-        <v>0</v>
-      </c>
-      <c r="K39" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L39" s="6"/>
       <c r="M39" s="6"/>
@@ -24779,37 +24782,35 @@
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="6">
-        <v>39</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="B40" s="6"/>
       <c r="C40" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E40" s="6">
-        <v>0</v>
-      </c>
-      <c r="F40" s="6">
-        <v>0</v>
-      </c>
-      <c r="G40" s="6">
-        <v>0</v>
-      </c>
-      <c r="H40" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K40" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L40" s="6"/>
       <c r="M40" s="6"/>
@@ -24818,37 +24819,35 @@
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="6">
-        <v>40</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="B41" s="6"/>
       <c r="C41" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="E41" s="6">
-        <v>0</v>
-      </c>
-      <c r="F41" s="6">
-        <v>0</v>
-      </c>
-      <c r="G41" s="6">
-        <v>0</v>
-      </c>
-      <c r="H41" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K41" s="6">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
@@ -24857,7 +24856,7 @@
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="6">
-        <v>42</v>
+        <v>81</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6" t="s">
@@ -24894,7 +24893,7 @@
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="6">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6" t="s">
@@ -24931,7 +24930,7 @@
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="6">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6" t="s">
@@ -24968,7 +24967,7 @@
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="6">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="6" t="s">
@@ -25005,7 +25004,7 @@
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="6">
-        <v>46</v>
+        <v>85</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6" t="s">
@@ -25042,7 +25041,7 @@
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="6">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6" t="s">
@@ -25079,7 +25078,7 @@
     </row>
     <row r="48" spans="1:15">
       <c r="A48" s="6">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
@@ -25116,7 +25115,7 @@
     </row>
     <row r="49" spans="1:15">
       <c r="A49" s="6">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6" t="s">
@@ -25153,7 +25152,7 @@
     </row>
     <row r="50" spans="1:15">
       <c r="A50" s="6">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6" t="s">
@@ -25190,7 +25189,7 @@
     </row>
     <row r="51" spans="1:15">
       <c r="A51" s="6">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="6" t="s">
@@ -25227,7 +25226,7 @@
     </row>
     <row r="52" spans="1:15">
       <c r="A52" s="6">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="6" t="s">
@@ -25264,7 +25263,7 @@
     </row>
     <row r="53" spans="1:15">
       <c r="A53" s="6">
-        <v>53</v>
+        <v>92</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6" t="s">
@@ -25301,7 +25300,7 @@
     </row>
     <row r="54" spans="1:15">
       <c r="A54" s="6">
-        <v>54</v>
+        <v>93</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6" t="s">
@@ -25338,7 +25337,7 @@
     </row>
     <row r="55" spans="1:15">
       <c r="A55" s="6">
-        <v>55</v>
+        <v>94</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="6" t="s">
@@ -25375,7 +25374,7 @@
     </row>
     <row r="56" spans="1:15">
       <c r="A56" s="6">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
@@ -25412,7 +25411,7 @@
     </row>
     <row r="57" spans="1:15">
       <c r="A57" s="6">
-        <v>57</v>
+        <v>96</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="6" t="s">
@@ -25449,7 +25448,7 @@
     </row>
     <row r="58" spans="1:15">
       <c r="A58" s="6">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="6" t="s">
@@ -25486,7 +25485,7 @@
     </row>
     <row r="59" spans="1:15">
       <c r="A59" s="6">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="6" t="s">
@@ -25523,7 +25522,7 @@
     </row>
     <row r="60" spans="1:15">
       <c r="A60" s="6">
-        <v>60</v>
+        <v>99</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6" t="s">
@@ -25560,7 +25559,7 @@
     </row>
     <row r="61" spans="1:15">
       <c r="A61" s="6">
-        <v>61</v>
+        <v>100</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6" t="s">
@@ -25596,9 +25595,7 @@
       <c r="O61" s="6"/>
     </row>
     <row r="62" spans="1:15">
-      <c r="A62" s="6">
-        <v>62</v>
-      </c>
+      <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6" t="s">
         <v>123</v>
@@ -25633,9 +25630,7 @@
       <c r="O62" s="6"/>
     </row>
     <row r="63" spans="1:15">
-      <c r="A63" s="6">
-        <v>63</v>
-      </c>
+      <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6" t="s">
         <v>123</v>
@@ -25670,9 +25665,7 @@
       <c r="O63" s="6"/>
     </row>
     <row r="64" spans="1:15">
-      <c r="A64" s="6">
-        <v>64</v>
-      </c>
+      <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6" t="s">
         <v>123</v>
@@ -25707,9 +25700,7 @@
       <c r="O64" s="6"/>
     </row>
     <row r="65" spans="1:15">
-      <c r="A65" s="6">
-        <v>65</v>
-      </c>
+      <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6" t="s">
         <v>123</v>
@@ -25744,9 +25735,7 @@
       <c r="O65" s="6"/>
     </row>
     <row r="66" spans="1:15">
-      <c r="A66" s="6">
-        <v>66</v>
-      </c>
+      <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6" t="s">
         <v>123</v>
@@ -25781,9 +25770,7 @@
       <c r="O66" s="6"/>
     </row>
     <row r="67" spans="1:15">
-      <c r="A67" s="6">
-        <v>67</v>
-      </c>
+      <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="6" t="s">
         <v>123</v>
@@ -25818,9 +25805,7 @@
       <c r="O67" s="6"/>
     </row>
     <row r="68" spans="1:15">
-      <c r="A68" s="6">
-        <v>68</v>
-      </c>
+      <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6" t="s">
         <v>123</v>
@@ -25855,9 +25840,7 @@
       <c r="O68" s="6"/>
     </row>
     <row r="69" spans="1:15">
-      <c r="A69" s="6">
-        <v>69</v>
-      </c>
+      <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="6" t="s">
         <v>123</v>
@@ -25892,9 +25875,7 @@
       <c r="O69" s="6"/>
     </row>
     <row r="70" spans="1:15">
-      <c r="A70" s="6">
-        <v>70</v>
-      </c>
+      <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="6" t="s">
         <v>123</v>
@@ -25929,9 +25910,7 @@
       <c r="O70" s="6"/>
     </row>
     <row r="71" spans="1:15">
-      <c r="A71" s="6">
-        <v>71</v>
-      </c>
+      <c r="A71" s="6"/>
       <c r="B71" s="6"/>
       <c r="C71" s="6" t="s">
         <v>123</v>
@@ -25966,9 +25945,7 @@
       <c r="O71" s="6"/>
     </row>
     <row r="72" spans="1:15">
-      <c r="A72" s="6">
-        <v>72</v>
-      </c>
+      <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6" t="s">
         <v>123</v>
@@ -26003,9 +25980,7 @@
       <c r="O72" s="6"/>
     </row>
     <row r="73" spans="1:15">
-      <c r="A73" s="6">
-        <v>73</v>
-      </c>
+      <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="6" t="s">
         <v>123</v>
@@ -26040,9 +26015,7 @@
       <c r="O73" s="6"/>
     </row>
     <row r="74" spans="1:15">
-      <c r="A74" s="6">
-        <v>74</v>
-      </c>
+      <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6" t="s">
         <v>123</v>
@@ -26077,9 +26050,7 @@
       <c r="O74" s="6"/>
     </row>
     <row r="75" spans="1:15">
-      <c r="A75" s="6">
-        <v>75</v>
-      </c>
+      <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6" t="s">
         <v>123</v>
@@ -26114,9 +26085,7 @@
       <c r="O75" s="6"/>
     </row>
     <row r="76" spans="1:15">
-      <c r="A76" s="6">
-        <v>76</v>
-      </c>
+      <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="6" t="s">
         <v>123</v>
@@ -26151,9 +26120,7 @@
       <c r="O76" s="6"/>
     </row>
     <row r="77" spans="1:15">
-      <c r="A77" s="6">
-        <v>77</v>
-      </c>
+      <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="6" t="s">
         <v>123</v>
@@ -26188,9 +26155,7 @@
       <c r="O77" s="6"/>
     </row>
     <row r="78" spans="1:15">
-      <c r="A78" s="6">
-        <v>78</v>
-      </c>
+      <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="6" t="s">
         <v>123</v>
@@ -26225,9 +26190,7 @@
       <c r="O78" s="6"/>
     </row>
     <row r="79" spans="1:15">
-      <c r="A79" s="6">
-        <v>79</v>
-      </c>
+      <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6" t="s">
         <v>123</v>
@@ -26262,9 +26225,7 @@
       <c r="O79" s="6"/>
     </row>
     <row r="80" spans="1:15">
-      <c r="A80" s="6">
-        <v>80</v>
-      </c>
+      <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6" t="s">
         <v>123</v>
@@ -26299,9 +26260,7 @@
       <c r="O80" s="6"/>
     </row>
     <row r="81" spans="1:15">
-      <c r="A81" s="6">
-        <v>81</v>
-      </c>
+      <c r="A81" s="6"/>
       <c r="B81" s="6"/>
       <c r="C81" s="6" t="s">
         <v>123</v>
@@ -26336,9 +26295,7 @@
       <c r="O81" s="6"/>
     </row>
     <row r="82" spans="1:15">
-      <c r="A82" s="6">
-        <v>82</v>
-      </c>
+      <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="6" t="s">
         <v>123</v>
@@ -26373,9 +26330,7 @@
       <c r="O82" s="6"/>
     </row>
     <row r="83" spans="1:15">
-      <c r="A83" s="6">
-        <v>83</v>
-      </c>
+      <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="6" t="s">
         <v>123</v>
@@ -26410,9 +26365,7 @@
       <c r="O83" s="6"/>
     </row>
     <row r="84" spans="1:15">
-      <c r="A84" s="6">
-        <v>84</v>
-      </c>
+      <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6" t="s">
         <v>123</v>
@@ -26447,9 +26400,7 @@
       <c r="O84" s="6"/>
     </row>
     <row r="85" spans="1:15">
-      <c r="A85" s="6">
-        <v>85</v>
-      </c>
+      <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="6" t="s">
         <v>123</v>
@@ -26484,9 +26435,7 @@
       <c r="O85" s="6"/>
     </row>
     <row r="86" spans="1:15">
-      <c r="A86" s="6">
-        <v>86</v>
-      </c>
+      <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="6" t="s">
         <v>123</v>
@@ -26521,9 +26470,7 @@
       <c r="O86" s="6"/>
     </row>
     <row r="87" spans="1:15">
-      <c r="A87" s="6">
-        <v>87</v>
-      </c>
+      <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="6" t="s">
         <v>123</v>
@@ -26558,9 +26505,7 @@
       <c r="O87" s="6"/>
     </row>
     <row r="88" spans="1:15">
-      <c r="A88" s="6">
-        <v>88</v>
-      </c>
+      <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6" t="s">
         <v>123</v>
@@ -26595,9 +26540,7 @@
       <c r="O88" s="6"/>
     </row>
     <row r="89" spans="1:15">
-      <c r="A89" s="6">
-        <v>89</v>
-      </c>
+      <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="6" t="s">
         <v>123</v>
@@ -26632,9 +26575,7 @@
       <c r="O89" s="6"/>
     </row>
     <row r="90" spans="1:15">
-      <c r="A90" s="6">
-        <v>90</v>
-      </c>
+      <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6" t="s">
         <v>123</v>
@@ -26669,9 +26610,7 @@
       <c r="O90" s="6"/>
     </row>
     <row r="91" spans="1:15">
-      <c r="A91" s="6">
-        <v>91</v>
-      </c>
+      <c r="A91" s="6"/>
       <c r="B91" s="6"/>
       <c r="C91" s="6" t="s">
         <v>123</v>
@@ -26706,9 +26645,7 @@
       <c r="O91" s="6"/>
     </row>
     <row r="92" spans="1:15">
-      <c r="A92" s="6">
-        <v>92</v>
-      </c>
+      <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6" t="s">
         <v>123</v>
@@ -26743,9 +26680,7 @@
       <c r="O92" s="6"/>
     </row>
     <row r="93" spans="1:15">
-      <c r="A93" s="6">
-        <v>93</v>
-      </c>
+      <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6" t="s">
         <v>123</v>
@@ -26780,9 +26715,7 @@
       <c r="O93" s="6"/>
     </row>
     <row r="94" spans="1:15">
-      <c r="A94" s="6">
-        <v>94</v>
-      </c>
+      <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6" t="s">
         <v>123</v>
@@ -26817,9 +26750,7 @@
       <c r="O94" s="6"/>
     </row>
     <row r="95" spans="1:15">
-      <c r="A95" s="6">
-        <v>95</v>
-      </c>
+      <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6" t="s">
         <v>123</v>
@@ -26854,9 +26785,7 @@
       <c r="O95" s="6"/>
     </row>
     <row r="96" spans="1:15">
-      <c r="A96" s="6">
-        <v>96</v>
-      </c>
+      <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="6" t="s">
         <v>123</v>
@@ -26891,9 +26820,7 @@
       <c r="O96" s="6"/>
     </row>
     <row r="97" spans="1:15">
-      <c r="A97" s="6">
-        <v>97</v>
-      </c>
+      <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="6" t="s">
         <v>123</v>
@@ -26928,9 +26855,7 @@
       <c r="O97" s="6"/>
     </row>
     <row r="98" spans="1:15">
-      <c r="A98" s="6">
-        <v>98</v>
-      </c>
+      <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="6" t="s">
         <v>123</v>
@@ -26965,9 +26890,7 @@
       <c r="O98" s="6"/>
     </row>
     <row r="99" spans="1:15">
-      <c r="A99" s="6">
-        <v>99</v>
-      </c>
+      <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6" t="s">
         <v>123</v>
@@ -27002,9 +26925,7 @@
       <c r="O99" s="6"/>
     </row>
     <row r="100" spans="1:15">
-      <c r="A100" s="6">
-        <v>100</v>
-      </c>
+      <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="6" t="s">
         <v>123</v>
@@ -27948,1373 +27869,8 @@
       <c r="N126" s="6"/>
       <c r="O126" s="6"/>
     </row>
-    <row r="127" spans="1:15">
-      <c r="A127" s="6"/>
-      <c r="B127" s="6"/>
-      <c r="C127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K127" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L127" s="6"/>
-      <c r="M127" s="6"/>
-      <c r="N127" s="6"/>
-      <c r="O127" s="6"/>
-    </row>
-    <row r="128" spans="1:15">
-      <c r="A128" s="6"/>
-      <c r="B128" s="6"/>
-      <c r="C128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K128" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L128" s="6"/>
-      <c r="M128" s="6"/>
-      <c r="N128" s="6"/>
-      <c r="O128" s="6"/>
-    </row>
-    <row r="129" spans="1:15">
-      <c r="A129" s="6"/>
-      <c r="B129" s="6"/>
-      <c r="C129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K129" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L129" s="6"/>
-      <c r="M129" s="6"/>
-      <c r="N129" s="6"/>
-      <c r="O129" s="6"/>
-    </row>
-    <row r="130" spans="1:15">
-      <c r="A130" s="6"/>
-      <c r="B130" s="6"/>
-      <c r="C130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K130" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L130" s="6"/>
-      <c r="M130" s="6"/>
-      <c r="N130" s="6"/>
-      <c r="O130" s="6"/>
-    </row>
-    <row r="131" spans="1:15">
-      <c r="A131" s="6"/>
-      <c r="B131" s="6"/>
-      <c r="C131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K131" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L131" s="6"/>
-      <c r="M131" s="6"/>
-      <c r="N131" s="6"/>
-      <c r="O131" s="6"/>
-    </row>
-    <row r="132" spans="1:15">
-      <c r="A132" s="6"/>
-      <c r="B132" s="6"/>
-      <c r="C132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K132" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L132" s="6"/>
-      <c r="M132" s="6"/>
-      <c r="N132" s="6"/>
-      <c r="O132" s="6"/>
-    </row>
-    <row r="133" spans="1:15">
-      <c r="A133" s="6"/>
-      <c r="B133" s="6"/>
-      <c r="C133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K133" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L133" s="6"/>
-      <c r="M133" s="6"/>
-      <c r="N133" s="6"/>
-      <c r="O133" s="6"/>
-    </row>
-    <row r="134" spans="1:15">
-      <c r="A134" s="6"/>
-      <c r="B134" s="6"/>
-      <c r="C134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K134" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L134" s="6"/>
-      <c r="M134" s="6"/>
-      <c r="N134" s="6"/>
-      <c r="O134" s="6"/>
-    </row>
-    <row r="135" spans="1:15">
-      <c r="A135" s="6"/>
-      <c r="B135" s="6"/>
-      <c r="C135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K135" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L135" s="6"/>
-      <c r="M135" s="6"/>
-      <c r="N135" s="6"/>
-      <c r="O135" s="6"/>
-    </row>
-    <row r="136" spans="1:15">
-      <c r="A136" s="6"/>
-      <c r="B136" s="6"/>
-      <c r="C136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K136" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L136" s="6"/>
-      <c r="M136" s="6"/>
-      <c r="N136" s="6"/>
-      <c r="O136" s="6"/>
-    </row>
-    <row r="137" spans="1:15">
-      <c r="A137" s="6"/>
-      <c r="B137" s="6"/>
-      <c r="C137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K137" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L137" s="6"/>
-      <c r="M137" s="6"/>
-      <c r="N137" s="6"/>
-      <c r="O137" s="6"/>
-    </row>
-    <row r="138" spans="1:15">
-      <c r="A138" s="6"/>
-      <c r="B138" s="6"/>
-      <c r="C138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K138" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L138" s="6"/>
-      <c r="M138" s="6"/>
-      <c r="N138" s="6"/>
-      <c r="O138" s="6"/>
-    </row>
-    <row r="139" spans="1:15">
-      <c r="A139" s="6"/>
-      <c r="B139" s="6"/>
-      <c r="C139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K139" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L139" s="6"/>
-      <c r="M139" s="6"/>
-      <c r="N139" s="6"/>
-      <c r="O139" s="6"/>
-    </row>
-    <row r="140" spans="1:15">
-      <c r="A140" s="6"/>
-      <c r="B140" s="6"/>
-      <c r="C140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K140" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L140" s="6"/>
-      <c r="M140" s="6"/>
-      <c r="N140" s="6"/>
-      <c r="O140" s="6"/>
-    </row>
-    <row r="141" spans="1:15">
-      <c r="A141" s="6"/>
-      <c r="B141" s="6"/>
-      <c r="C141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K141" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L141" s="6"/>
-      <c r="M141" s="6"/>
-      <c r="N141" s="6"/>
-      <c r="O141" s="6"/>
-    </row>
-    <row r="142" spans="1:15">
-      <c r="A142" s="6"/>
-      <c r="B142" s="6"/>
-      <c r="C142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K142" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L142" s="6"/>
-      <c r="M142" s="6"/>
-      <c r="N142" s="6"/>
-      <c r="O142" s="6"/>
-    </row>
-    <row r="143" spans="1:15">
-      <c r="A143" s="6"/>
-      <c r="B143" s="6"/>
-      <c r="C143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K143" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L143" s="6"/>
-      <c r="M143" s="6"/>
-      <c r="N143" s="6"/>
-      <c r="O143" s="6"/>
-    </row>
-    <row r="144" spans="1:15">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
-      <c r="C144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K144" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L144" s="6"/>
-      <c r="M144" s="6"/>
-      <c r="N144" s="6"/>
-      <c r="O144" s="6"/>
-    </row>
-    <row r="145" spans="1:15">
-      <c r="A145" s="6"/>
-      <c r="B145" s="6"/>
-      <c r="C145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K145" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L145" s="6"/>
-      <c r="M145" s="6"/>
-      <c r="N145" s="6"/>
-      <c r="O145" s="6"/>
-    </row>
-    <row r="146" spans="1:15">
-      <c r="A146" s="6"/>
-      <c r="B146" s="6"/>
-      <c r="C146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K146" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L146" s="6"/>
-      <c r="M146" s="6"/>
-      <c r="N146" s="6"/>
-      <c r="O146" s="6"/>
-    </row>
-    <row r="147" spans="1:15">
-      <c r="A147" s="6"/>
-      <c r="B147" s="6"/>
-      <c r="C147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K147" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L147" s="6"/>
-      <c r="M147" s="6"/>
-      <c r="N147" s="6"/>
-      <c r="O147" s="6"/>
-    </row>
-    <row r="148" spans="1:15">
-      <c r="A148" s="6"/>
-      <c r="B148" s="6"/>
-      <c r="C148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K148" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L148" s="6"/>
-      <c r="M148" s="6"/>
-      <c r="N148" s="6"/>
-      <c r="O148" s="6"/>
-    </row>
-    <row r="149" spans="1:15">
-      <c r="A149" s="6"/>
-      <c r="B149" s="6"/>
-      <c r="C149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K149" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L149" s="6"/>
-      <c r="M149" s="6"/>
-      <c r="N149" s="6"/>
-      <c r="O149" s="6"/>
-    </row>
-    <row r="150" spans="1:15">
-      <c r="A150" s="6"/>
-      <c r="B150" s="6"/>
-      <c r="C150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K150" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L150" s="6"/>
-      <c r="M150" s="6"/>
-      <c r="N150" s="6"/>
-      <c r="O150" s="6"/>
-    </row>
-    <row r="151" spans="1:15">
-      <c r="A151" s="6"/>
-      <c r="B151" s="6"/>
-      <c r="C151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K151" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L151" s="6"/>
-      <c r="M151" s="6"/>
-      <c r="N151" s="6"/>
-      <c r="O151" s="6"/>
-    </row>
-    <row r="152" spans="1:15">
-      <c r="A152" s="6"/>
-      <c r="B152" s="6"/>
-      <c r="C152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K152" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L152" s="6"/>
-      <c r="M152" s="6"/>
-      <c r="N152" s="6"/>
-      <c r="O152" s="6"/>
-    </row>
-    <row r="153" spans="1:15">
-      <c r="A153" s="6"/>
-      <c r="B153" s="6"/>
-      <c r="C153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K153" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L153" s="6"/>
-      <c r="M153" s="6"/>
-      <c r="N153" s="6"/>
-      <c r="O153" s="6"/>
-    </row>
-    <row r="154" spans="1:15">
-      <c r="A154" s="6"/>
-      <c r="B154" s="6"/>
-      <c r="C154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K154" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L154" s="6"/>
-      <c r="M154" s="6"/>
-      <c r="N154" s="6"/>
-      <c r="O154" s="6"/>
-    </row>
-    <row r="155" spans="1:15">
-      <c r="A155" s="6"/>
-      <c r="B155" s="6"/>
-      <c r="C155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K155" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L155" s="6"/>
-      <c r="M155" s="6"/>
-      <c r="N155" s="6"/>
-      <c r="O155" s="6"/>
-    </row>
-    <row r="156" spans="1:15">
-      <c r="A156" s="6"/>
-      <c r="B156" s="6"/>
-      <c r="C156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K156" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L156" s="6"/>
-      <c r="M156" s="6"/>
-      <c r="N156" s="6"/>
-      <c r="O156" s="6"/>
-    </row>
-    <row r="157" spans="1:15">
-      <c r="A157" s="6"/>
-      <c r="B157" s="6"/>
-      <c r="C157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K157" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L157" s="6"/>
-      <c r="M157" s="6"/>
-      <c r="N157" s="6"/>
-      <c r="O157" s="6"/>
-    </row>
-    <row r="158" spans="1:15">
-      <c r="A158" s="6"/>
-      <c r="B158" s="6"/>
-      <c r="C158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K158" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L158" s="6"/>
-      <c r="M158" s="6"/>
-      <c r="N158" s="6"/>
-      <c r="O158" s="6"/>
-    </row>
-    <row r="159" spans="1:15">
-      <c r="A159" s="6"/>
-      <c r="B159" s="6"/>
-      <c r="C159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K159" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L159" s="6"/>
-      <c r="M159" s="6"/>
-      <c r="N159" s="6"/>
-      <c r="O159" s="6"/>
-    </row>
-    <row r="160" spans="1:15">
-      <c r="A160" s="6"/>
-      <c r="B160" s="6"/>
-      <c r="C160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K160" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L160" s="6"/>
-      <c r="M160" s="6"/>
-      <c r="N160" s="6"/>
-      <c r="O160" s="6"/>
-    </row>
-    <row r="161" spans="1:15">
-      <c r="A161" s="6"/>
-      <c r="B161" s="6"/>
-      <c r="C161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K161" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L161" s="6"/>
-      <c r="M161" s="6"/>
-      <c r="N161" s="6"/>
-      <c r="O161" s="6"/>
-    </row>
-    <row r="162" spans="1:15">
-      <c r="A162" s="6"/>
-      <c r="B162" s="6"/>
-      <c r="C162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K162" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L162" s="6"/>
-      <c r="M162" s="6"/>
-      <c r="N162" s="6"/>
-      <c r="O162" s="6"/>
-    </row>
-    <row r="163" spans="1:15">
-      <c r="A163" s="6"/>
-      <c r="B163" s="6"/>
-      <c r="C163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K163" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L163" s="6"/>
-      <c r="M163" s="6"/>
-      <c r="N163" s="6"/>
-      <c r="O163" s="6"/>
-    </row>
-    <row r="164" spans="1:15">
-      <c r="A164" s="6"/>
-      <c r="B164" s="6"/>
-      <c r="C164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K164" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L164" s="6"/>
-      <c r="M164" s="6"/>
-      <c r="N164" s="6"/>
-      <c r="O164" s="6"/>
-    </row>
-    <row r="165" spans="1:15">
-      <c r="A165" s="6"/>
-      <c r="B165" s="6"/>
-      <c r="C165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="G165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="H165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="K165" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="L165" s="6"/>
-      <c r="M165" s="6"/>
-      <c r="N165" s="6"/>
-      <c r="O165" s="6"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P100">
+  <conditionalFormatting sqref="A2:P3 A13:P61 A4:B12 E4:P12">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
@@ -29345,7 +27901,7 @@
           <x14:formula1>
             <xm:f>_helper!$A$1:$A$15</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B100</xm:sqref>
+          <xm:sqref>B2:B61</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
18 06 20 05 26
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A62CA6-1AB1-4931-9288-DDA198331371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F681613A-A145-44B4-A8F2-C4978EFD9692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_helper" sheetId="3" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2753" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2799" uniqueCount="212">
   <si>
     <t>id</t>
   </si>
@@ -682,6 +682,48 @@
   </si>
   <si>
     <t>/</t>
+  </si>
+  <si>
+    <t>Диаметр отвечает за размер пикселя: чем больше диаметр иглы, тем крупнее получается пиксель; стандартные обозначения — 0,25; 0,30; 0,35.</t>
+  </si>
+  <si>
+    <t>Количество игл — цифры после диаметра обозначают количество игл одного диаметра в спайке; стандартные обозначения: 01, 03, 05.</t>
+  </si>
+  <si>
+    <t>Конфигурация </t>
+  </si>
+  <si>
+    <t>Конфигурация — это тип спайки игл в картридже, от которой зависит, какой рисунок из пикселей будет оставлять модуль; основные типы конфигурации для перманента.</t>
+  </si>
+  <si>
+    <t>RL (round liner) - иглы плотно спаяны в пучок на самом конце. Для четких контуров или прокраса на тонкой, фарфоровой или возрастной коже.</t>
+  </si>
+  <si>
+    <t>RS (round shader) - иглы спаяны параллельно друг другу пучок более широкий, пиксель более рассыпчатый. Так же можно использовать в работе с прокрасом на тонкой и возрастной коже.</t>
+  </si>
+  <si>
+    <t>M (magnum) - иглы спаянные в ряд имеют прямой, плоский срез. Все иглы в спайке одинаковой длины. Не используются в ПМ.</t>
+  </si>
+  <si>
+    <t>RM (round magnum) - спайка игл в форме полумесяца.</t>
+  </si>
+  <si>
+    <t>Заточка</t>
+  </si>
+  <si>
+    <t>LT (long taper) - самая длинная и острая заточка. Прокол маленького диаметра отлично подходит для фиксации эскиза.</t>
+  </si>
+  <si>
+    <t>MT ( medium taper) - заточка средней длинны, самая универсальная подходит как для фиксации эскиза так и для прокраса на любой зоне перманента.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST ( short taper) - самая короткая и «тупая» заточка. </t>
+  </si>
+  <si>
+    <t>Конусность — это длина острой части иглы, которую делят на несколько типов.</t>
+  </si>
+  <si>
+    <t>Дополнением к данным заточкам существуют текстурированные иглы, обозначаются на маркировке дополнительной приставкой “T” ( например 3001 RLLT-T ). Такие иглы имеют рельефное покрытие, за счет своей структуры берут на себя больше пигмента в результате чего в коже так же остается больше пигмента. Стоит учесть текстурированные иглы не подойдут на чувстельную и тонкую кожу, так как являются более травматичными.</t>
   </si>
 </sst>
 </file>
@@ -24230,25 +24272,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A43:P43">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="76" priority="1">
       <formula>ISNUMBER(SEARCH("text",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="75" priority="2">
       <formula>ISNUMBER(SEARCH("title",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="74" priority="3">
       <formula>ISNUMBER(SEARCH("hero",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="73" priority="4">
       <formula>ISNUMBER(SEARCH("card",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="72" priority="5">
       <formula>ISNUMBER(SEARCH("carousel",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="71" priority="6">
       <formula>ISNUMBER(SEARCH("video",$B43))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="70" priority="7">
       <formula>ISNUMBER(SEARCH("image",$B43))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -28914,48 +28956,48 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P3 A47:P62 A5:B46 E5:P46">
-    <cfRule type="expression" dxfId="76" priority="8">
+    <cfRule type="expression" dxfId="69" priority="8">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="9">
+    <cfRule type="expression" dxfId="68" priority="9">
       <formula>ISNUMBER(SEARCH("title",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="10">
+    <cfRule type="expression" dxfId="67" priority="10">
       <formula>ISNUMBER(SEARCH("hero",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="11">
+    <cfRule type="expression" dxfId="66" priority="11">
       <formula>ISNUMBER(SEARCH("card",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="12">
+    <cfRule type="expression" dxfId="65" priority="12">
       <formula>ISNUMBER(SEARCH("carousel",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="13">
+    <cfRule type="expression" dxfId="64" priority="13">
       <formula>ISNUMBER(SEARCH("video",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="14">
+    <cfRule type="expression" dxfId="63" priority="14">
       <formula>ISNUMBER(SEARCH("image",$B2))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:P4">
-    <cfRule type="expression" dxfId="69" priority="1">
+    <cfRule type="expression" dxfId="62" priority="1">
       <formula>ISNUMBER(SEARCH("text",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="2">
+    <cfRule type="expression" dxfId="61" priority="2">
       <formula>ISNUMBER(SEARCH("title",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="3">
+    <cfRule type="expression" dxfId="60" priority="3">
       <formula>ISNUMBER(SEARCH("hero",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="4">
+    <cfRule type="expression" dxfId="59" priority="4">
       <formula>ISNUMBER(SEARCH("card",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="5">
+    <cfRule type="expression" dxfId="58" priority="5">
       <formula>ISNUMBER(SEARCH("carousel",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="6">
+    <cfRule type="expression" dxfId="57" priority="6">
       <formula>ISNUMBER(SEARCH("video",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="7">
+    <cfRule type="expression" dxfId="56" priority="7">
       <formula>ISNUMBER(SEARCH("image",$B4))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35184,140 +35226,140 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:D2 A16:D16 E3:P3 A3:B3 A18:P102 E17:P17 A17:B17 A5:B15 E5:P15 G2:P2 G16:P16">
-    <cfRule type="expression" dxfId="62" priority="36">
+    <cfRule type="expression" dxfId="55" priority="36">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="37">
+    <cfRule type="expression" dxfId="54" priority="37">
       <formula>ISNUMBER(SEARCH("title",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="38">
+    <cfRule type="expression" dxfId="53" priority="38">
       <formula>ISNUMBER(SEARCH("hero",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="39">
+    <cfRule type="expression" dxfId="52" priority="39">
       <formula>ISNUMBER(SEARCH("card",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="40">
+    <cfRule type="expression" dxfId="51" priority="40">
       <formula>ISNUMBER(SEARCH("carousel",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="41">
+    <cfRule type="expression" dxfId="50" priority="41">
       <formula>ISNUMBER(SEARCH("video",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="42">
+    <cfRule type="expression" dxfId="49" priority="42">
       <formula>ISNUMBER(SEARCH("image",$B2))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:P4">
-    <cfRule type="expression" dxfId="55" priority="29">
+    <cfRule type="expression" dxfId="48" priority="29">
       <formula>ISNUMBER(SEARCH("text",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="30">
+    <cfRule type="expression" dxfId="47" priority="30">
       <formula>ISNUMBER(SEARCH("title",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="31">
+    <cfRule type="expression" dxfId="46" priority="31">
       <formula>ISNUMBER(SEARCH("hero",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="32">
+    <cfRule type="expression" dxfId="45" priority="32">
       <formula>ISNUMBER(SEARCH("card",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="33">
+    <cfRule type="expression" dxfId="44" priority="33">
       <formula>ISNUMBER(SEARCH("carousel",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="34">
+    <cfRule type="expression" dxfId="43" priority="34">
       <formula>ISNUMBER(SEARCH("video",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="49" priority="35">
+    <cfRule type="expression" dxfId="42" priority="35">
       <formula>ISNUMBER(SEARCH("image",$B4))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="expression" dxfId="48" priority="22">
+    <cfRule type="expression" dxfId="41" priority="22">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="23">
+    <cfRule type="expression" dxfId="40" priority="23">
       <formula>ISNUMBER(SEARCH("title",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="24">
+    <cfRule type="expression" dxfId="39" priority="24">
       <formula>ISNUMBER(SEARCH("hero",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="25">
+    <cfRule type="expression" dxfId="38" priority="25">
       <formula>ISNUMBER(SEARCH("card",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="26">
+    <cfRule type="expression" dxfId="37" priority="26">
       <formula>ISNUMBER(SEARCH("carousel",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="27">
+    <cfRule type="expression" dxfId="36" priority="27">
       <formula>ISNUMBER(SEARCH("video",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="28">
+    <cfRule type="expression" dxfId="35" priority="28">
       <formula>ISNUMBER(SEARCH("image",$B2))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2">
-    <cfRule type="expression" dxfId="41" priority="15">
+    <cfRule type="expression" dxfId="34" priority="15">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="16">
+    <cfRule type="expression" dxfId="33" priority="16">
       <formula>ISNUMBER(SEARCH("title",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="17">
+    <cfRule type="expression" dxfId="32" priority="17">
       <formula>ISNUMBER(SEARCH("hero",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="18">
+    <cfRule type="expression" dxfId="31" priority="18">
       <formula>ISNUMBER(SEARCH("card",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="19">
+    <cfRule type="expression" dxfId="30" priority="19">
       <formula>ISNUMBER(SEARCH("carousel",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="20">
+    <cfRule type="expression" dxfId="29" priority="20">
       <formula>ISNUMBER(SEARCH("video",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="21">
+    <cfRule type="expression" dxfId="28" priority="21">
       <formula>ISNUMBER(SEARCH("image",$B2))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="expression" dxfId="34" priority="8">
+    <cfRule type="expression" dxfId="27" priority="8">
       <formula>ISNUMBER(SEARCH("text",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="9">
+    <cfRule type="expression" dxfId="26" priority="9">
       <formula>ISNUMBER(SEARCH("title",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="10">
+    <cfRule type="expression" dxfId="25" priority="10">
       <formula>ISNUMBER(SEARCH("hero",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="11">
+    <cfRule type="expression" dxfId="24" priority="11">
       <formula>ISNUMBER(SEARCH("card",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="12">
+    <cfRule type="expression" dxfId="23" priority="12">
       <formula>ISNUMBER(SEARCH("carousel",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="13">
+    <cfRule type="expression" dxfId="22" priority="13">
       <formula>ISNUMBER(SEARCH("video",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="14">
+    <cfRule type="expression" dxfId="21" priority="14">
       <formula>ISNUMBER(SEARCH("image",$B16))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F16">
-    <cfRule type="expression" dxfId="27" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>ISNUMBER(SEARCH("text",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>ISNUMBER(SEARCH("title",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>ISNUMBER(SEARCH("hero",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>ISNUMBER(SEARCH("card",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="5">
+    <cfRule type="expression" dxfId="16" priority="5">
       <formula>ISNUMBER(SEARCH("carousel",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="6">
+    <cfRule type="expression" dxfId="15" priority="6">
       <formula>ISNUMBER(SEARCH("video",$B16))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="7">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>ISNUMBER(SEARCH("image",$B16))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35455,10 +35497,10 @@
       <c r="B3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" t="s">
         <v>182</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" t="s">
         <v>182</v>
       </c>
       <c r="E3" s="6">
@@ -35517,6 +35559,8 @@
       <c r="B4" s="6" t="s">
         <v>65</v>
       </c>
+      <c r="C4"/>
+      <c r="D4"/>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="6">
@@ -35525,10 +35569,10 @@
       <c r="B5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" t="s">
         <v>183</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" t="s">
         <v>183</v>
       </c>
       <c r="E5" s="6">
@@ -35587,10 +35631,10 @@
       <c r="B6" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" t="s">
         <v>184</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" t="s">
         <v>184</v>
       </c>
       <c r="E6" s="6">
@@ -35649,10 +35693,10 @@
       <c r="B7" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" t="s">
         <v>185</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" t="s">
         <v>185</v>
       </c>
       <c r="E7" s="6">
@@ -35711,10 +35755,10 @@
       <c r="B8" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" t="s">
         <v>186</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" t="s">
         <v>186</v>
       </c>
       <c r="E8" s="6">
@@ -35773,10 +35817,10 @@
       <c r="B9" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" t="s">
         <v>187</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" t="s">
         <v>187</v>
       </c>
       <c r="E9" s="6">
@@ -35832,1116 +35876,1096 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6" t="str">
-        <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D10" s="6" t="str">
+      <c r="B10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E10" s="6" t="str">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>images/example_ru.jpg</v>
       </c>
       <c r="F10" s="6" t="str">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G10" s="6" t="str">
+        <v>images/example_ua.jpg</v>
+      </c>
+      <c r="G10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H10" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I10" s="6" t="str">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>↑ Квадратное изображение (300×300px, по центру)</v>
       </c>
       <c r="J10" s="6" t="str">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K10" s="6" t="str">
+        <v>↑ Квадратне зображення (300×300px, по центру)</v>
+      </c>
+      <c r="K10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L10" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M10" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="M10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N10" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="N10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="O10" s="6" t="str">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P10" s="6" t="str">
+        <v>contain</v>
+      </c>
+      <c r="P10" s="6">
         <f>IF($B10="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B10,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6" t="str">
-        <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D11" s="6" t="str">
-        <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E11" s="6" t="str">
+      <c r="B11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" t="s">
+        <v>198</v>
+      </c>
+      <c r="E11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P11" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P11" s="6">
         <f>IF($B11="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B11,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6" t="str">
-        <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D12" s="6" t="str">
-        <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E12" s="6" t="str">
+      <c r="B12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>199</v>
+      </c>
+      <c r="D12" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P12" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P12" s="6">
         <f>IF($B12="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B12,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6" t="str">
-        <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D13" s="6" t="str">
-        <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+      <c r="B13" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="E13" s="6" t="str">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>images/example_ru.jpg</v>
       </c>
       <c r="F13" s="6" t="str">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G13" s="6" t="str">
+        <v>images/example_ua.jpg</v>
+      </c>
+      <c r="G13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H13" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I13" s="6" t="str">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>↑ Квадратное изображение (300×300px, по центру)</v>
       </c>
       <c r="J13" s="6" t="str">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K13" s="6" t="str">
+        <v>↑ Квадратне зображення (300×300px, по центру)</v>
+      </c>
+      <c r="K13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L13" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M13" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="M13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N13" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="N13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="str">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P13" s="6" t="str">
+        <v>contain</v>
+      </c>
+      <c r="P13" s="6">
         <f>IF($B13="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B13,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6" t="str">
-        <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D14" s="6" t="str">
-        <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E14" s="6" t="str">
+      <c r="B14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" t="s">
+        <v>200</v>
+      </c>
+      <c r="D14" t="s">
+        <v>200</v>
+      </c>
+      <c r="E14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P14" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6">
         <f>IF($B14="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B14,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6" t="str">
-        <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D15" s="6" t="str">
-        <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E15" s="6" t="str">
+      <c r="B15" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D15" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P15" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P15" s="6">
         <f>IF($B15="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B15,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6" t="str">
-        <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D16" s="6" t="str">
-        <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E16" s="6" t="str">
+      <c r="B16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D16" t="s">
+        <v>202</v>
+      </c>
+      <c r="E16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P16" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P16" s="6">
         <f>IF($B16="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B16,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:16">
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6" t="str">
-        <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D17" s="6" t="str">
-        <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E17" s="6" t="str">
+      <c r="B17" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D17" t="s">
+        <v>203</v>
+      </c>
+      <c r="E17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P17" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P17" s="6">
         <f>IF($B17="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B17,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6" t="str">
-        <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D18" s="6" t="str">
-        <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E18" s="6" t="str">
+      <c r="B18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" t="s">
+        <v>204</v>
+      </c>
+      <c r="D18" t="s">
+        <v>204</v>
+      </c>
+      <c r="E18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P18" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P18" s="6">
         <f>IF($B18="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B18,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6" t="str">
-        <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D19" s="6" t="str">
-        <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E19" s="6" t="str">
+      <c r="B19" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
+        <v>205</v>
+      </c>
+      <c r="D19" t="s">
+        <v>205</v>
+      </c>
+      <c r="E19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P19" s="6">
         <f>IF($B19="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B19,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="6">
-        <v>18</v>
-      </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6" t="str">
-        <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D20" s="6" t="str">
-        <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>11</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="E20" s="6" t="str">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>images/example_ru.jpg</v>
       </c>
       <c r="F20" s="6" t="str">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G20" s="6" t="str">
+        <v>images/example_ua.jpg</v>
+      </c>
+      <c r="G20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I20" s="6" t="str">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>↑ Квадратное изображение (300×300px, по центру)</v>
       </c>
       <c r="J20" s="6" t="str">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K20" s="6" t="str">
+        <v>↑ Квадратне зображення (300×300px, по центру)</v>
+      </c>
+      <c r="K20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M20" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="M20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N20" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="N20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="O20" s="6" t="str">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P20" s="6" t="str">
+        <v>contain</v>
+      </c>
+      <c r="P20" s="6">
         <f>IF($B20="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B20,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6" t="str">
-        <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D21" s="6" t="str">
-        <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E21" s="6" t="str">
+      <c r="B21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>206</v>
+      </c>
+      <c r="D21" t="s">
+        <v>206</v>
+      </c>
+      <c r="E21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P21" s="6">
         <f>IF($B21="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B21,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6" t="str">
-        <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D22" s="6" t="str">
-        <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E22" s="6" t="str">
+      <c r="B22" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" t="s">
+        <v>210</v>
+      </c>
+      <c r="D22" t="s">
+        <v>210</v>
+      </c>
+      <c r="E22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P22" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P22" s="6">
         <f>IF($B22="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B22,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:16">
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6" t="str">
-        <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D23" s="6" t="str">
-        <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E23" s="6" t="str">
+      <c r="B23" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P23" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P23" s="6">
         <f>IF($B23="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B23,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6" t="str">
-        <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D24" s="6" t="str">
-        <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E24" s="6" t="str">
+      <c r="B24" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P24" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P24" s="6">
         <f>IF($B24="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B24,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6" t="str">
-        <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D25" s="6" t="str">
-        <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E25" s="6" t="str">
+      <c r="B25" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P25" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P25" s="6">
         <f>IF($B25="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B25,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6" t="str">
-        <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D26" s="6" t="str">
-        <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E26" s="6" t="str">
+      <c r="B26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="E26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="I26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="J26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="O26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P26" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="P26" s="6">
         <f>IF($B26="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B26,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="6">
-        <v>25</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6" t="str">
-        <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$C:$C,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D27" s="6" t="str">
-        <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$D:$D,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>11</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="E27" s="6" t="str">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$E:$E,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>images/example_ru.jpg</v>
       </c>
       <c r="F27" s="6" t="str">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$F:$F,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G27" s="6" t="str">
+        <v>images/example_ua.jpg</v>
+      </c>
+      <c r="G27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$G:$G,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="H27" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$H:$H,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I27" s="6" t="str">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$I:$I,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>↑ Квадратное изображение (300×300px, по центру)</v>
       </c>
       <c r="J27" s="6" t="str">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$J:$J,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="K27" s="6" t="str">
+        <v>↑ Квадратне зображення (300×300px, по центру)</v>
+      </c>
+      <c r="K27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$K:$K,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="L27" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$L:$L,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="M27" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="M27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$M:$M,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="N27" s="6" t="str">
+        <v>300</v>
+      </c>
+      <c r="N27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$N:$N,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="O27" s="6" t="str">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$O:$O,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
-      </c>
-      <c r="P27" s="6" t="str">
+        <v>contain</v>
+      </c>
+      <c r="P27" s="6">
         <f>IF($B27="","",IFERROR(INDEX('Типы элементов'!$P:$P,MATCH($B27,'Типы элементов'!$B:$B,0)),""))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -41595,56 +41619,56 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P3 A5:P102">
-    <cfRule type="expression" dxfId="20" priority="8">
+  <conditionalFormatting sqref="A2:P3 A5:P10 E11:P11 D12:P12 C13:P14 A11:B19 E15:P19 A20:P20 A21:B22 E21:P22 A23:P102">
+    <cfRule type="expression" dxfId="13" priority="8">
       <formula>ISNUMBER(SEARCH("text",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="9">
+    <cfRule type="expression" dxfId="12" priority="9">
       <formula>ISNUMBER(SEARCH("title",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="10">
+    <cfRule type="expression" dxfId="11" priority="10">
       <formula>ISNUMBER(SEARCH("hero",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>ISNUMBER(SEARCH("card",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="12">
+    <cfRule type="expression" dxfId="9" priority="12">
       <formula>ISNUMBER(SEARCH("carousel",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="13">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>ISNUMBER(SEARCH("video",$B2))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>ISNUMBER(SEARCH("image",$B2))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:P4">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>ISNUMBER(SEARCH("text",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>ISNUMBER(SEARCH("title",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>ISNUMBER(SEARCH("hero",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>ISNUMBER(SEARCH("card",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>ISNUMBER(SEARCH("carousel",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>ISNUMBER(SEARCH("video",$B4))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>ISNUMBER(SEARCH("image",$B4))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{B6596A43-5FC2-403F-9232-D44EA528B072}">
           <x14:formula1>
             <xm:f>_helper!$A$1:$A$15</xm:f>

</xml_diff>

<commit_message>
huge changes was made
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58F9D35-61B3-42B5-B3C9-A55B2F359F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAF9F18-9F2C-47DF-A537-83CC5F5D9BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_empty" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="82">
   <si>
     <t>id</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>images/hero.jpg</t>
-  </si>
-  <si>
-    <t>w=1200;h=520;resizeMode=cover</t>
   </si>
   <si>
     <t>eyebrow</t>
@@ -1105,28 +1102,25 @@
       <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="L2" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
-        <v>18</v>
-      </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1134,19 +1128,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>21</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1154,19 +1148,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>26</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>27</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -1174,19 +1168,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>30</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>32</v>
-      </c>
-      <c r="F6" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -1194,22 +1188,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
         <v>34</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" t="s">
         <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>35</v>
-      </c>
-      <c r="L7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -1217,22 +1211,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" t="s">
         <v>38</v>
-      </c>
-      <c r="D8" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" t="s">
-        <v>38</v>
-      </c>
-      <c r="L8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -1240,34 +1234,34 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
         <v>41</v>
       </c>
-      <c r="D9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>42</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>43</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>44</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>45</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>46</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>47</v>
-      </c>
-      <c r="K9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1275,19 +1269,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
         <v>49</v>
       </c>
-      <c r="C10" t="s">
-        <v>50</v>
-      </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1295,22 +1289,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>52</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>53</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>54</v>
       </c>
-      <c r="F11" t="s">
+      <c r="K11" t="s">
         <v>55</v>
-      </c>
-      <c r="K11" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1318,19 +1312,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>58</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>59</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>60</v>
-      </c>
-      <c r="F12" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1338,22 +1332,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
         <v>62</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>63</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>65</v>
       </c>
-      <c r="F13" t="s">
+      <c r="K13" t="s">
         <v>66</v>
-      </c>
-      <c r="K13" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1361,34 +1355,34 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
         <v>68</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>69</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>70</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>72</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>73</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>74</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>75</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>76</v>
-      </c>
-      <c r="K14" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1492,7 +1486,7 @@
         <v/>
       </c>
       <c r="N2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1540,7 +1534,7 @@
         <v/>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1588,7 +1582,7 @@
         <v/>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -6097,12 +6091,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B2,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="L2" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B2,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>w=1200;h=520;resizeMode=cover</v>
-      </c>
       <c r="N2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -6110,7 +6100,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B3,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6153,7 +6143,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -6161,7 +6151,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B4,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6204,7 +6194,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -6212,7 +6202,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B5,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6260,7 +6250,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B6,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6308,7 +6298,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6343,7 +6333,7 @@
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
       <c r="K7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L7">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6355,7 +6345,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6390,7 +6380,7 @@
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
       <c r="K8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L8">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6402,7 +6392,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6437,7 +6427,7 @@
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
       <c r="K9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L9">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6449,7 +6439,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -6484,7 +6474,7 @@
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
       <c r="K10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L10">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -10731,12 +10721,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B2,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="L2" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B2,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>w=1200;h=520;resizeMode=cover</v>
-      </c>
       <c r="N2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -10744,7 +10730,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B3,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -10787,7 +10773,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -10795,7 +10781,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B4,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -10838,7 +10824,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -10846,7 +10832,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B5,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -10894,7 +10880,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="4"/>
@@ -10920,17 +10906,13 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B6,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="L6" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B6,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>w=600;h=400;resizeMode=contain</v>
-      </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -10978,7 +10960,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11026,7 +11008,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11074,7 +11056,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11118,7 +11100,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C11" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B11,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11162,7 +11144,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B12,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11206,7 +11188,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C13" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B13,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11250,7 +11232,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B14,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11298,7 +11280,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B15,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11346,7 +11328,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11394,19 +11376,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G17">
         <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B17,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11428,17 +11410,13 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B17,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="L17" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B17,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>w=400;h=225;resizeMode=contain</v>
-      </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C18" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B18,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11473,7 +11451,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L18">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B18,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -11484,48 +11462,41 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
       <c r="C19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>images/animation.gif</v>
+        <v/>
       </c>
       <c r="D19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>images/animation.gif</v>
+        <v/>
       </c>
       <c r="E19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>images/animation.gif</v>
+        <v/>
       </c>
       <c r="F19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>images/animation.gif</v>
-      </c>
-      <c r="G19">
+        <v/>
+      </c>
+      <c r="G19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="H19">
+        <v/>
+      </c>
+      <c r="H19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="I19">
+        <v/>
+      </c>
+      <c r="I19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="J19">
+        <v/>
+      </c>
+      <c r="J19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="K19">
+        <v/>
+      </c>
+      <c r="K19" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="L19" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B19,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>w=400;h=225;resizeMode=contain</v>
+        <v/>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -15304,62 +15275,62 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
before text color change
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36365BC-54FD-4925-8525-2829A852A149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF898AA-E185-454A-AF6E-4987DFFBAD05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="87">
   <si>
     <t>id</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>3. Замените пример своим текстом</t>
+  </si>
+  <si>
+    <t>/skin</t>
   </si>
   <si>
     <t>spacer</t>
@@ -1509,7 +1512,7 @@
         <v>13</v>
       </c>
       <c r="L2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1799,37 +1802,37 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -8897,9 +8900,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
-      <c r="K7" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>/lesson-example</v>
+      <c r="K7" t="s">
+        <v>80</v>
       </c>
       <c r="L7">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B7,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -8945,9 +8947,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
-      <c r="K8" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>/lesson-example</v>
+      <c r="K8" t="s">
+        <v>80</v>
       </c>
       <c r="L8">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B8,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -8993,9 +8994,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
-      <c r="K9" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>/lesson-example</v>
+      <c r="K9" t="s">
+        <v>80</v>
       </c>
       <c r="L9">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -9041,9 +9041,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v>Kartenbeschreibung auf Deutsch</v>
       </c>
-      <c r="K10" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>/lesson-example</v>
+      <c r="K10" t="s">
+        <v>80</v>
       </c>
       <c r="L10">
         <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B10,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -15334,7 +15333,7 @@
       <formula>$B2="languageSwitcher"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" error="Выберите значение из списка" prompt="Выберите тип элемента" sqref="B2:B11" xr:uid="{25F84185-1A22-4266-9C7D-B5D3601F8D72}">
       <formula1>TypeList</formula1>
     </dataValidation>
@@ -15342,7 +15341,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{2DD349C1-D3B3-4AB3-94AF-1F183742C58F}">
           <x14:formula1>
             <xm:f>OFFSET('Колонки и примеры'!$B$2,0,0,COUNTA('Колонки и примеры'!$B:$B)-1,1)</xm:f>
@@ -15756,7 +15755,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B9,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16092,23 +16091,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>Секция</v>
-      </c>
-      <c r="D16" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>Секция</v>
-      </c>
-      <c r="E16" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>Section</v>
-      </c>
-      <c r="F16" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v>Abschnitt</v>
+        <v>81</v>
       </c>
       <c r="G16" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B16,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -22249,7 +22232,7 @@
       <formula>$B9="languageSwitcher"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" error="Выберите значение из списка" prompt="Выберите тип элемента" sqref="B10:B21 B2:B8" xr:uid="{F856262F-FF67-4496-9DA8-9A87E6D409D2}">
       <formula1>TypeList</formula1>
     </dataValidation>
@@ -22257,7 +22240,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{C0B528CB-38BC-4839-B6C2-1B9407FD1CF3}">
           <x14:formula1>
             <xm:f>OFFSET('Колонки и примеры'!$B$2,0,0,COUNTA('Колонки и примеры'!$B:$B)-1,1)</xm:f>

</xml_diff>

<commit_message>
timer done befor checklist
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0CC59B5-23E1-4F0D-9078-370192439BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D4D8E2-A0DE-423A-B801-B124998928FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_empty" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="141">
   <si>
     <t>id</t>
   </si>
@@ -454,6 +454,18 @@
   <si>
     <t>2</t>
   </si>
+  <si>
+    <t>timer</t>
+  </si>
+  <si>
+    <t>seconds=180</t>
+  </si>
+  <si>
+    <t>seconds=60</t>
+  </si>
+  <si>
+    <t>seconds=30</t>
+  </si>
 </sst>
 </file>
 
@@ -529,8 +541,80 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE0F7FA"/>
-          <bgColor rgb="FFE0F7FA"/>
+          <fgColor rgb="FFE8F4FD"/>
+          <bgColor rgb="FFE8F4FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF4E5"/>
+          <bgColor rgb="FFFFF4E5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF7EA"/>
+          <bgColor rgb="FFEAF7EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3E8FD"/>
+          <bgColor rgb="FFF3E8FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+          <bgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEF7E7"/>
+          <bgColor rgb="FFEEF7E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF9DB"/>
+          <bgColor rgb="FFFFF9DB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE8E6"/>
+          <bgColor rgb="FFFCE8E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE6F4EA"/>
+          <bgColor rgb="FFE6F4EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF1F3F4"/>
+          <bgColor rgb="FFF1F3F4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -545,24 +629,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF1F3F4"/>
-          <bgColor rgb="FFF1F3F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE6F4EA"/>
-          <bgColor rgb="FFE6F4EA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE8E6"/>
-          <bgColor rgb="FFFCE8E6"/>
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -577,168 +645,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFF9DB"/>
-          <bgColor rgb="FFFFF9DB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFEEF7E7"/>
           <bgColor rgb="FFEEF7E7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFDECEC"/>
-          <bgColor rgb="FFFDECEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF3E8FD"/>
-          <bgColor rgb="FFF3E8FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAF7EA"/>
-          <bgColor rgb="FFEAF7EA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF4E5"/>
-          <bgColor rgb="FFFFF4E5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE8F4FD"/>
-          <bgColor rgb="FFE8F4FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE0F7FA"/>
-          <bgColor rgb="FFE0F7FA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF3E5F5"/>
-          <bgColor rgb="FFF3E5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF1F3F4"/>
-          <bgColor rgb="FFF1F3F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE6F4EA"/>
-          <bgColor rgb="FFE6F4EA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE8E6"/>
-          <bgColor rgb="FFFCE8E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE8F0FE"/>
-          <bgColor rgb="FFE8F0FE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF9DB"/>
-          <bgColor rgb="FFFFF9DB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEF7E7"/>
-          <bgColor rgb="FFEEF7E7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFDECEC"/>
-          <bgColor rgb="FFFDECEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF3E8FD"/>
-          <bgColor rgb="FFF3E8FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAF7EA"/>
-          <bgColor rgb="FFEAF7EA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF4E5"/>
-          <bgColor rgb="FFFFF4E5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE8F4FD"/>
-          <bgColor rgb="FFE8F4FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE0F7FA"/>
-          <bgColor rgb="FFE0F7FA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -809,14 +717,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEEF7E7"/>
-          <bgColor rgb="FFEEF7E7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFDECEC"/>
           <bgColor rgb="FFFDECEC"/>
         </patternFill>
@@ -851,6 +751,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFE8F4FD"/>
           <bgColor rgb="FFE8F4FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -913,14 +821,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEEF7E7"/>
-          <bgColor rgb="FFEEF7E7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFDECEC"/>
           <bgColor rgb="FFFDECEC"/>
         </patternFill>
@@ -955,6 +855,118 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFE8F4FD"/>
           <bgColor rgb="FFE8F4FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEF7E7"/>
+          <bgColor rgb="FFEEF7E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0F7FA"/>
+          <bgColor rgb="FFE0F7FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE8F4FD"/>
+          <bgColor rgb="FFE8F4FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF4E5"/>
+          <bgColor rgb="FFFFF4E5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF7EA"/>
+          <bgColor rgb="FFEAF7EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3E8FD"/>
+          <bgColor rgb="FFF3E8FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+          <bgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEF7E7"/>
+          <bgColor rgb="FFEEF7E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF9DB"/>
+          <bgColor rgb="FFFFF9DB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE8F0FE"/>
+          <bgColor rgb="FFE8F0FE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE8E6"/>
+          <bgColor rgb="FFFCE8E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE6F4EA"/>
+          <bgColor rgb="FFE6F4EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF1F3F4"/>
+          <bgColor rgb="FFF1F3F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3E5F5"/>
+          <bgColor rgb="FFF3E5F5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1601,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC7D9512-43B5-4068-A86B-B844ABA8B948}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1996,7 +2008,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.75">
+    <row r="16" spans="1:12" ht="15.75" customHeight="1">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2032,6 +2044,44 @@
       </c>
       <c r="L16" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" t="s">
+        <v>86</v>
+      </c>
+      <c r="G17" t="s">
+        <v>86</v>
+      </c>
+      <c r="H17" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" t="s">
+        <v>86</v>
+      </c>
+      <c r="J17" t="s">
+        <v>86</v>
+      </c>
+      <c r="K17" t="s">
+        <v>86</v>
+      </c>
+      <c r="L17" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -15351,7 +15401,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A10:L99 A2:A9 C2:L9">
+  <conditionalFormatting sqref="A2:A9 C2:L9 A10:L99">
     <cfRule type="expression" dxfId="81" priority="14">
       <formula>$B2="spacer"</formula>
     </cfRule>
@@ -16461,6 +16511,9 @@
       <c r="A22">
         <v>22</v>
       </c>
+      <c r="B22" t="s">
+        <v>137</v>
+      </c>
       <c r="C22" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B22,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
@@ -16497,15 +16550,17 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B22,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
-      <c r="L22" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B22,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+      <c r="L22" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23">
         <v>23</v>
       </c>
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
       <c r="C23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
@@ -16542,9 +16597,8 @@
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
-      <c r="L23" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+      <c r="L23" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -22113,68 +22167,68 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A21:L100 A2:A20 C2:L20">
-    <cfRule type="expression" dxfId="54" priority="42">
-      <formula>$B2="spacer"</formula>
+  <conditionalFormatting sqref="A2:A20 C2:L20 A21:L100">
+    <cfRule type="expression" dxfId="54" priority="55">
+      <formula>$B2="languageSwitcher"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="43">
+    <cfRule type="expression" dxfId="53" priority="54">
+      <formula>$B2="navigationButtons"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="53">
+      <formula>$B2="item"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="51" priority="52">
+      <formula>$B2="link"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="50" priority="51">
+      <formula>$B2="video"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="50">
+      <formula>$B2="card"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="49">
+      <formula>$B2="gif"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="47" priority="48">
+      <formula>$B2="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="47">
+      <formula>$B2="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="46">
+      <formula>$B2="subtitle"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="45">
+      <formula>$B2="title"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="44">
+      <formula>$B2="eyebrow"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="42" priority="43">
       <formula>$B2="heroImage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="44">
-      <formula>$B2="eyebrow"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="51" priority="45">
-      <formula>$B2="title"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="50" priority="46">
-      <formula>$B2="subtitle"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="49" priority="47">
-      <formula>$B2="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="48" priority="48">
-      <formula>$B2="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="47" priority="49">
-      <formula>$B2="gif"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="46" priority="50">
-      <formula>$B2="card"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="45" priority="51">
-      <formula>$B2="video"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="44" priority="52">
-      <formula>$B2="link"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="43" priority="53">
-      <formula>$B2="item"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="54">
-      <formula>$B2="navigationButtons"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="41" priority="55">
-      <formula>$B2="languageSwitcher"</formula>
+    <cfRule type="expression" dxfId="41" priority="42">
+      <formula>$B2="spacer"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B14">
-    <cfRule type="expression" dxfId="40" priority="2">
+    <cfRule type="expression" dxfId="40" priority="7">
+      <formula>$B2="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="2">
       <formula>$B2="heroImage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="3">
+    <cfRule type="expression" dxfId="38" priority="3">
       <formula>$B2="eyebrow"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="4">
+    <cfRule type="expression" dxfId="37" priority="4">
       <formula>$B2="title"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="5">
+    <cfRule type="expression" dxfId="36" priority="5">
       <formula>$B2="subtitle"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="6">
+    <cfRule type="expression" dxfId="35" priority="6">
       <formula>$B2="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="35" priority="7">
-      <formula>$B2="image"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="34" priority="8">
       <formula>$B2="gif"</formula>
@@ -22204,88 +22258,88 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="26" priority="28">
+    <cfRule type="expression" dxfId="26" priority="29">
+      <formula>$B15="heroImage"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="30">
+      <formula>$B15="eyebrow"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="31">
+      <formula>$B15="title"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="32">
+      <formula>$B15="subtitle"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="33">
+      <formula>$B15="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="35">
+      <formula>$B15="gif"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="36">
+      <formula>$B15="card"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="37">
+      <formula>$B15="video"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="38">
+      <formula>$B15="link"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="39">
+      <formula>$B15="item"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="40">
+      <formula>$B15="navigationButtons"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="41">
+      <formula>$B15="languageSwitcher"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="28">
       <formula>$B15="spacer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="29">
-      <formula>$B15="heroImage"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="30">
-      <formula>$B15="eyebrow"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="23" priority="31">
-      <formula>$B15="title"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="32">
-      <formula>$B15="subtitle"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="21" priority="33">
-      <formula>$B15="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="20" priority="34">
+    <cfRule type="expression" dxfId="13" priority="34">
       <formula>$B15="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="35">
-      <formula>$B15="gif"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="36">
-      <formula>$B15="card"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="37">
-      <formula>$B15="video"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="38">
-      <formula>$B15="link"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="39">
-      <formula>$B15="item"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="40">
-      <formula>$B15="navigationButtons"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="41">
-      <formula>$B15="languageSwitcher"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:B20">
-    <cfRule type="expression" dxfId="12" priority="15">
-      <formula>$B16="heroImage"</formula>
+    <cfRule type="expression" dxfId="12" priority="22">
+      <formula>$B16="card"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="16">
-      <formula>$B16="eyebrow"</formula>
+    <cfRule type="expression" dxfId="11" priority="27">
+      <formula>$B16="languageSwitcher"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="17">
-      <formula>$B16="title"</formula>
+    <cfRule type="expression" dxfId="10" priority="26">
+      <formula>$B16="navigationButtons"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="18">
-      <formula>$B16="subtitle"</formula>
+    <cfRule type="expression" dxfId="9" priority="25">
+      <formula>$B16="item"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="19">
-      <formula>$B16="text"</formula>
+    <cfRule type="expression" dxfId="8" priority="24">
+      <formula>$B16="link"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="20">
-      <formula>$B16="image"</formula>
+    <cfRule type="expression" dxfId="7" priority="23">
+      <formula>$B16="video"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="21">
       <formula>$B16="gif"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="22">
-      <formula>$B16="card"</formula>
+    <cfRule type="expression" dxfId="5" priority="20">
+      <formula>$B16="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="23">
-      <formula>$B16="video"</formula>
+    <cfRule type="expression" dxfId="4" priority="19">
+      <formula>$B16="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="24">
-      <formula>$B16="link"</formula>
+    <cfRule type="expression" dxfId="3" priority="18">
+      <formula>$B16="subtitle"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="25">
-      <formula>$B16="item"</formula>
+    <cfRule type="expression" dxfId="2" priority="17">
+      <formula>$B16="title"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="26">
-      <formula>$B16="navigationButtons"</formula>
+    <cfRule type="expression" dxfId="1" priority="16">
+      <formula>$B16="eyebrow"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="27">
-      <formula>$B16="languageSwitcher"</formula>
+    <cfRule type="expression" dxfId="0" priority="15">
+      <formula>$B16="heroImage"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>

<commit_message>
before vis change after checlist add
</commit_message>
<xml_diff>
--- a/src/content/content.xlsx
+++ b/src/content/content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eugsinsh gmail drive\NA\na_mi_pmu\src\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D4D8E2-A0DE-423A-B801-B124998928FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815E7F47-9615-493F-BB6C-CBC8531A70C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,8 @@
     <sheet name="index" sheetId="15" r:id="rId4"/>
     <sheet name="skin" sheetId="16" r:id="rId5"/>
     <sheet name="quiz1" sheetId="17" r:id="rId6"/>
-    <sheet name="lists" sheetId="4" state="hidden" r:id="rId7"/>
+    <sheet name="checklist1" sheetId="18" r:id="rId7"/>
+    <sheet name="lists" sheetId="4" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="TypeList">lists!$A$1:$A$13</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="167">
   <si>
     <t>id</t>
   </si>
@@ -461,10 +462,88 @@
     <t>seconds=180</t>
   </si>
   <si>
-    <t>seconds=60</t>
+    <t>seconds=30</t>
   </si>
   <si>
-    <t>seconds=30</t>
+    <t>checklist</t>
+  </si>
+  <si>
+    <t>Список задач</t>
+  </si>
+  <si>
+    <t>Checklist</t>
+  </si>
+  <si>
+    <t>Checkliste</t>
+  </si>
+  <si>
+    <t>checklist1</t>
+  </si>
+  <si>
+    <t>Чеклист підготовки</t>
+  </si>
+  <si>
+    <t>Чеклист подготовки</t>
+  </si>
+  <si>
+    <t>Preparation checklist</t>
+  </si>
+  <si>
+    <t>Vorbereitungs-Checkliste</t>
+  </si>
+  <si>
+    <t>Выполните эти пункты перед началом занятия.</t>
+  </si>
+  <si>
+    <t>Complete these steps before you start.</t>
+  </si>
+  <si>
+    <t>Führen Sie diese Schritte vor dem Start aus.</t>
+  </si>
+  <si>
+    <t>Проверить оборудование</t>
+  </si>
+  <si>
+    <t>Check the equipment</t>
+  </si>
+  <si>
+    <t>Geräte prüfen</t>
+  </si>
+  <si>
+    <t>Подготовить рабочее место</t>
+  </si>
+  <si>
+    <t>Prepare the workspace</t>
+  </si>
+  <si>
+    <t>Arbeitsplatz vorbereiten</t>
+  </si>
+  <si>
+    <t>Прочитать технику выполнения</t>
+  </si>
+  <si>
+    <t>Read the procedure</t>
+  </si>
+  <si>
+    <t>Verfahren lesen</t>
+  </si>
+  <si>
+    <t>Собрать необходимые материалы</t>
+  </si>
+  <si>
+    <t>Gather the required materials</t>
+  </si>
+  <si>
+    <t>Benötigte Materialien sammeln</t>
+  </si>
+  <si>
+    <t>Проверить план урока</t>
+  </si>
+  <si>
+    <t>Review the lesson plan</t>
+  </si>
+  <si>
+    <t>Lehrplan überprüfen</t>
   </si>
 </sst>
 </file>
@@ -1214,15 +1293,19 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF1F3F4"/>
-          <bgColor rgb="FFF1F3F4"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE6F4EA"/>
-          <bgColor rgb="FFE6F4EA"/>
+          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1230,7 +1313,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFCE8E6"/>
-          <bgColor rgb="FFFCE8E6"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1238,7 +1321,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE8F0FE"/>
-          <bgColor rgb="FFE8F0FE"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1246,7 +1329,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF9DB"/>
-          <bgColor rgb="FFFFF9DB"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1254,15 +1337,19 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEF7E7"/>
-          <bgColor rgb="FFEEF7E7"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFDECEC"/>
-          <bgColor rgb="FFFDECEC"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1270,11 +1357,15 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF3E8FD"/>
-          <bgColor rgb="FFF3E8FD"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEAF7EA"/>
@@ -1613,7 +1704,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC7D9512-43B5-4068-A86B-B844ABA8B948}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -2082,6 +2173,44 @@
       </c>
       <c r="L17" t="s">
         <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" t="s">
+        <v>142</v>
+      </c>
+      <c r="F18" t="s">
+        <v>143</v>
+      </c>
+      <c r="G18" t="s">
+        <v>86</v>
+      </c>
+      <c r="H18" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" t="s">
+        <v>86</v>
+      </c>
+      <c r="J18" t="s">
+        <v>86</v>
+      </c>
+      <c r="K18" t="s">
+        <v>144</v>
+      </c>
+      <c r="L18" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -15509,7 +15638,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF4888ED-D378-4723-8571-C65D6731076B}">
-  <dimension ref="A1:N150"/>
+  <dimension ref="A1:N149"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -16551,31 +16680,31 @@
         <v/>
       </c>
       <c r="L22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+        <v>Список задач</v>
       </c>
       <c r="D23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+        <v>Список задач</v>
       </c>
       <c r="E23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+        <v>Checklist</v>
       </c>
       <c r="F23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
+        <v>Checkliste</v>
       </c>
       <c r="G23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16595,15 +16724,16 @@
       </c>
       <c r="K23" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L23" t="s">
-        <v>139</v>
+        <v>checklist1</v>
+      </c>
+      <c r="L23" t="str">
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B23,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <v/>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="A24">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C24" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B24,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16648,7 +16778,7 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C25" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B25,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16693,7 +16823,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C26" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B26,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16738,7 +16868,7 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C27" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B27,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16783,7 +16913,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C28" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B28,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16828,7 +16958,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C29" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B29,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16873,7 +17003,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B30,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16918,7 +17048,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C31" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B31,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -16963,7 +17093,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C32" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B32,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17008,7 +17138,7 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C33" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B33,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17053,7 +17183,7 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C34" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B34,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17098,7 +17228,7 @@
     </row>
     <row r="35" spans="1:12">
       <c r="A35">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C35" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B35,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17143,7 +17273,7 @@
     </row>
     <row r="36" spans="1:12">
       <c r="A36">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C36" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B36,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17188,7 +17318,7 @@
     </row>
     <row r="37" spans="1:12">
       <c r="A37">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C37" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B37,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17233,7 +17363,7 @@
     </row>
     <row r="38" spans="1:12">
       <c r="A38">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C38" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B38,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17278,7 +17408,7 @@
     </row>
     <row r="39" spans="1:12">
       <c r="A39">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C39" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B39,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17323,7 +17453,7 @@
     </row>
     <row r="40" spans="1:12">
       <c r="A40">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C40" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B40,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17368,7 +17498,7 @@
     </row>
     <row r="41" spans="1:12">
       <c r="A41">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C41" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B41,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17413,7 +17543,7 @@
     </row>
     <row r="42" spans="1:12">
       <c r="A42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C42" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B42,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17458,7 +17588,7 @@
     </row>
     <row r="43" spans="1:12">
       <c r="A43">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C43" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B43,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17503,7 +17633,7 @@
     </row>
     <row r="44" spans="1:12">
       <c r="A44">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C44" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B44,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17548,7 +17678,7 @@
     </row>
     <row r="45" spans="1:12">
       <c r="A45">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C45" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B45,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17593,7 +17723,7 @@
     </row>
     <row r="46" spans="1:12">
       <c r="A46">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C46" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B46,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17638,7 +17768,7 @@
     </row>
     <row r="47" spans="1:12">
       <c r="A47">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C47" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B47,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17683,7 +17813,7 @@
     </row>
     <row r="48" spans="1:12">
       <c r="A48">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C48" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B48,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17728,7 +17858,7 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C49" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B49,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17773,7 +17903,7 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C50" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B50,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17818,7 +17948,7 @@
     </row>
     <row r="51" spans="1:12">
       <c r="A51">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C51" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B51,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17863,7 +17993,7 @@
     </row>
     <row r="52" spans="1:12">
       <c r="A52">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C52" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B52,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17908,7 +18038,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C53" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B53,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17953,7 +18083,7 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C54" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B54,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -17998,7 +18128,7 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C55" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B55,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18043,7 +18173,7 @@
     </row>
     <row r="56" spans="1:12">
       <c r="A56">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C56" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B56,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18088,7 +18218,7 @@
     </row>
     <row r="57" spans="1:12">
       <c r="A57">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C57" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B57,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18133,7 +18263,7 @@
     </row>
     <row r="58" spans="1:12">
       <c r="A58">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C58" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B58,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18178,7 +18308,7 @@
     </row>
     <row r="59" spans="1:12">
       <c r="A59">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C59" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B59,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18223,7 +18353,7 @@
     </row>
     <row r="60" spans="1:12">
       <c r="A60">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C60" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B60,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18268,7 +18398,7 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C61" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B61,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18313,7 +18443,7 @@
     </row>
     <row r="62" spans="1:12">
       <c r="A62">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C62" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B62,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18358,7 +18488,7 @@
     </row>
     <row r="63" spans="1:12">
       <c r="A63">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C63" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B63,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18403,7 +18533,7 @@
     </row>
     <row r="64" spans="1:12">
       <c r="A64">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C64" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B64,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18448,7 +18578,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C65" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B65,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18493,7 +18623,7 @@
     </row>
     <row r="66" spans="1:12">
       <c r="A66">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C66" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B66,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18538,7 +18668,7 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C67" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B67,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18583,7 +18713,7 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C68" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B68,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18628,7 +18758,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C69" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B69,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18673,7 +18803,7 @@
     </row>
     <row r="70" spans="1:12">
       <c r="A70">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C70" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B70,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18718,7 +18848,7 @@
     </row>
     <row r="71" spans="1:12">
       <c r="A71">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C71" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B71,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18763,7 +18893,7 @@
     </row>
     <row r="72" spans="1:12">
       <c r="A72">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C72" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B72,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18808,7 +18938,7 @@
     </row>
     <row r="73" spans="1:12">
       <c r="A73">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C73" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B73,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18853,7 +18983,7 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C74" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B74,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18898,7 +19028,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C75" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B75,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18943,7 +19073,7 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C76" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B76,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -18988,7 +19118,7 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C77" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B77,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19033,7 +19163,7 @@
     </row>
     <row r="78" spans="1:12">
       <c r="A78">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C78" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B78,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19078,7 +19208,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C79" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B79,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19123,7 +19253,7 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C80" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B80,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19168,7 +19298,7 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C81" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B81,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19213,7 +19343,7 @@
     </row>
     <row r="82" spans="1:12">
       <c r="A82">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C82" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B82,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19258,7 +19388,7 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C83" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B83,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19303,7 +19433,7 @@
     </row>
     <row r="84" spans="1:12">
       <c r="A84">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C84" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B84,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19348,7 +19478,7 @@
     </row>
     <row r="85" spans="1:12">
       <c r="A85">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C85" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B85,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19393,7 +19523,7 @@
     </row>
     <row r="86" spans="1:12">
       <c r="A86">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C86" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B86,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19438,7 +19568,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C87" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B87,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19483,7 +19613,7 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C88" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B88,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19528,7 +19658,7 @@
     </row>
     <row r="89" spans="1:12">
       <c r="A89">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C89" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B89,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19573,7 +19703,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C90" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B90,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19618,7 +19748,7 @@
     </row>
     <row r="91" spans="1:12">
       <c r="A91">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C91" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B91,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19663,7 +19793,7 @@
     </row>
     <row r="92" spans="1:12">
       <c r="A92">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C92" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B92,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19708,7 +19838,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C93" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B93,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19753,7 +19883,7 @@
     </row>
     <row r="94" spans="1:12">
       <c r="A94">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C94" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B94,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19798,7 +19928,7 @@
     </row>
     <row r="95" spans="1:12">
       <c r="A95">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C95" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B95,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19843,7 +19973,7 @@
     </row>
     <row r="96" spans="1:12">
       <c r="A96">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C96" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B96,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19888,7 +20018,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C97" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B97,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19933,7 +20063,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C98" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B98,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -19978,7 +20108,7 @@
     </row>
     <row r="99" spans="1:12">
       <c r="A99">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C99" t="str">
         <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
@@ -20022,2152 +20152,2107 @@
       </c>
     </row>
     <row r="100" spans="1:12">
-      <c r="A100">
-        <v>100</v>
-      </c>
       <c r="C100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L100" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="101" spans="1:12">
       <c r="C101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L101" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="102" spans="1:12">
       <c r="C102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L102" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="103" spans="1:12">
       <c r="C103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L103" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="104" spans="1:12">
       <c r="C104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L104" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="105" spans="1:12">
       <c r="C105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L105" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="106" spans="1:12">
       <c r="C106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L106" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="107" spans="1:12">
       <c r="C107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L107" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="108" spans="1:12">
       <c r="C108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L108" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="109" spans="1:12">
       <c r="C109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L109" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="110" spans="1:12">
       <c r="C110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L110" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="111" spans="1:12">
       <c r="C111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L111" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="112" spans="1:12">
       <c r="C112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L112" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="113" spans="3:12">
       <c r="C113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L113" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="114" spans="3:12">
       <c r="C114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L114" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="115" spans="3:12">
       <c r="C115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L115" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="116" spans="3:12">
       <c r="C116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L116" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="117" spans="3:12">
       <c r="C117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L117" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="118" spans="3:12">
       <c r="C118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L118" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="119" spans="3:12">
       <c r="C119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L119" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="120" spans="3:12">
       <c r="C120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L120" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="121" spans="3:12">
       <c r="C121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L121" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="122" spans="3:12">
       <c r="C122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L122" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="123" spans="3:12">
       <c r="C123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L123" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="124" spans="3:12">
       <c r="C124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L124" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="125" spans="3:12">
       <c r="C125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L125" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="126" spans="3:12">
       <c r="C126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L126" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="127" spans="3:12">
       <c r="C127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L127" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="128" spans="3:12">
       <c r="C128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L128" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="129" spans="3:12">
       <c r="C129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L129" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="130" spans="3:12">
       <c r="C130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L130" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="131" spans="3:12">
       <c r="C131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L131" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="132" spans="3:12">
       <c r="C132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L132" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="133" spans="3:12">
       <c r="C133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L133" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="134" spans="3:12">
       <c r="C134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L134" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="135" spans="3:12">
       <c r="C135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L135" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="136" spans="3:12">
       <c r="C136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L136" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="137" spans="3:12">
       <c r="C137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L137" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="138" spans="3:12">
       <c r="C138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L138" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="139" spans="3:12">
       <c r="C139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L139" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="140" spans="3:12">
       <c r="C140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L140" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="141" spans="3:12">
       <c r="C141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L141" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="142" spans="3:12">
       <c r="C142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L142" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="143" spans="3:12">
       <c r="C143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L143" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="144" spans="3:12">
       <c r="C144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L144" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="145" spans="3:12">
       <c r="C145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L145" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="146" spans="3:12">
       <c r="C146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L146" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="147" spans="3:12">
       <c r="C147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L147" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="148" spans="3:12">
       <c r="C148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L148" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="149" spans="3:12">
       <c r="C149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="D149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="E149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="F149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="G149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="H149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="I149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="J149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="K149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
       <c r="L149" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="150" spans="3:12">
-      <c r="C150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!C:C,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!D:D,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!E:E,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!F:F,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!G:G,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!H:H,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!I:I,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!J:J,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!K:K,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L150" t="str">
-        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B100,'Колонки и примеры'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('Колонки и примеры'!L:L,MATCH($B99,'Колонки и примеры'!$B:$B,0)),"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A20 C2:L20 A21:L100">
+  <conditionalFormatting sqref="A2:A20 C2:L20 A21:L99">
     <cfRule type="expression" dxfId="54" priority="55">
       <formula>$B2="languageSwitcher"</formula>
     </cfRule>
@@ -22358,7 +22443,7 @@
           <x14:formula1>
             <xm:f>OFFSET('Колонки и примеры'!$B$2,0,0,COUNTA('Колонки и примеры'!$B:$B)-1,1)</xm:f>
           </x14:formula1>
-          <xm:sqref>B21:B999</xm:sqref>
+          <xm:sqref>B21:B998</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -22644,6 +22729,326 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538C8DA0-65DE-444B-AB8F-96D225EBA84C}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="6.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="3" customWidth="1"/>
+    <col min="3" max="6" width="41" style="3" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>